<commit_message>
Updated 834 converted files
</commit_message>
<xml_diff>
--- a/converted_files/834/X220-add-dependent-(full-time-student)-to-existing-enrollment.xlsx
+++ b/converted_files/834/X220-add-dependent-(full-time-student)-to-existing-enrollment.xlsx
@@ -59,7 +59,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:PD2"/>
+  <dimension ref="A1:PO2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -220,1945 +220,2000 @@
       </c>
       <c r="AF1" s="3" t="inlineStr">
         <is>
+          <t>MedicarePlanCode</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>MedicareEligibilityReasonCode</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
           <t>CobraEventCode</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>EmploymentStatusCode</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>StudentStatusCode</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>HandicapIndicator</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
+        <is>
+          <t>DeathDate</t>
+        </is>
+      </c>
+      <c r="AM1" s="3" t="inlineStr">
         <is>
           <t>ConfidentialityCode</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>BirthSequenceNumber</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AO1" s="3" t="inlineStr">
         <is>
           <t>Identifier</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AP1" s="3" t="inlineStr">
         <is>
           <t>GroupOrPolicyNumber</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier1QualifierCode</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier1Identification</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier2QualifierCode</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier2Identification</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier3QualifierCode</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier3Identification</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier4QualifierCode</t>
         </is>
       </c>
-      <c r="AU1" s="3" t="inlineStr">
+      <c r="AX1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier4Identification</t>
         </is>
       </c>
-      <c r="AV1" s="3" t="inlineStr">
+      <c r="AY1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier5QualifierCode</t>
         </is>
       </c>
-      <c r="AW1" s="3" t="inlineStr">
+      <c r="AZ1" s="3" t="inlineStr">
         <is>
           <t>SupplementalIdentifier5Identification</t>
         </is>
       </c>
-      <c r="AX1" s="3" t="inlineStr">
+      <c r="BA1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate1QualifierCode</t>
         </is>
       </c>
-      <c r="AY1" s="3" t="inlineStr">
+      <c r="BB1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate1Date</t>
         </is>
       </c>
-      <c r="AZ1" s="3" t="inlineStr">
+      <c r="BC1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate2QualifierCode</t>
         </is>
       </c>
-      <c r="BA1" s="3" t="inlineStr">
+      <c r="BD1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate2Date</t>
         </is>
       </c>
-      <c r="BB1" s="3" t="inlineStr">
+      <c r="BE1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate3QualifierCode</t>
         </is>
       </c>
-      <c r="BC1" s="3" t="inlineStr">
+      <c r="BF1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate3Date</t>
         </is>
       </c>
-      <c r="BD1" s="3" t="inlineStr">
+      <c r="BG1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate4QualifierCode</t>
         </is>
       </c>
-      <c r="BE1" s="3" t="inlineStr">
+      <c r="BH1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate4Date</t>
         </is>
       </c>
-      <c r="BF1" s="3" t="inlineStr">
+      <c r="BI1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate5QualifierCode</t>
         </is>
       </c>
-      <c r="BG1" s="3" t="inlineStr">
+      <c r="BJ1" s="3" t="inlineStr">
         <is>
           <t>StatusInfoEffectiveDate5Date</t>
         </is>
       </c>
-      <c r="BH1" s="3" t="inlineStr">
+      <c r="BK1" s="3" t="inlineStr">
         <is>
           <t>MemberEntityRole</t>
         </is>
       </c>
-      <c r="BI1" s="3" t="inlineStr">
+      <c r="BL1" s="3" t="inlineStr">
         <is>
           <t>MemberIdentificationType</t>
         </is>
       </c>
-      <c r="BJ1" s="3" t="inlineStr">
+      <c r="BM1" s="3" t="inlineStr">
         <is>
           <t>MemberIdentifier</t>
         </is>
       </c>
-      <c r="BK1" s="3" t="inlineStr">
+      <c r="BN1" s="3" t="inlineStr">
         <is>
           <t>MemberTaxId</t>
         </is>
       </c>
-      <c r="BL1" s="3" t="inlineStr">
+      <c r="BO1" s="3" t="inlineStr">
         <is>
           <t>MemberLastName</t>
         </is>
       </c>
-      <c r="BM1" s="3" t="inlineStr">
+      <c r="BP1" s="3" t="inlineStr">
         <is>
           <t>MemberFirstName</t>
         </is>
       </c>
-      <c r="BN1" s="3" t="inlineStr">
+      <c r="BQ1" s="3" t="inlineStr">
         <is>
           <t>MemberMiddleName</t>
         </is>
       </c>
-      <c r="BO1" s="3" t="inlineStr">
+      <c r="BR1" s="3" t="inlineStr">
         <is>
           <t>MemberBirthDate</t>
         </is>
       </c>
-      <c r="BP1" s="3" t="inlineStr">
+      <c r="BS1" s="3" t="inlineStr">
         <is>
           <t>MemberGender</t>
         </is>
       </c>
-      <c r="BQ1" s="3" t="inlineStr">
+      <c r="BT1" s="3" t="inlineStr">
         <is>
           <t>MemberAddressLine</t>
         </is>
       </c>
-      <c r="BR1" s="3" t="inlineStr">
+      <c r="BU1" s="3" t="inlineStr">
         <is>
           <t>MemberAddressLine2</t>
         </is>
       </c>
-      <c r="BS1" s="3" t="inlineStr">
+      <c r="BV1" s="3" t="inlineStr">
         <is>
           <t>MemberAddressCity</t>
         </is>
       </c>
-      <c r="BT1" s="3" t="inlineStr">
+      <c r="BW1" s="3" t="inlineStr">
         <is>
           <t>MemberAddressStateCode</t>
         </is>
       </c>
-      <c r="BU1" s="3" t="inlineStr">
+      <c r="BX1" s="3" t="inlineStr">
         <is>
           <t>MemberAddressZipCode</t>
         </is>
       </c>
-      <c r="BV1" s="3" t="inlineStr">
+      <c r="BY1" s="3" t="inlineStr">
         <is>
           <t>MemberContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="BW1" s="3" t="inlineStr">
+      <c r="BZ1" s="3" t="inlineStr">
         <is>
           <t>MemberContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="BX1" s="3" t="inlineStr">
+      <c r="CA1" s="3" t="inlineStr">
         <is>
           <t>MemberContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="BY1" s="3" t="inlineStr">
+      <c r="CB1" s="3" t="inlineStr">
         <is>
           <t>MemberContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="BZ1" s="3" t="inlineStr">
+      <c r="CC1" s="3" t="inlineStr">
         <is>
           <t>MemberMaritalStatusCode</t>
         </is>
       </c>
-      <c r="CA1" s="3" t="inlineStr">
-        <is>
-          <t>MemberEthnicityCode</t>
-        </is>
-      </c>
-      <c r="CB1" s="3" t="inlineStr">
+      <c r="CD1" s="3" t="inlineStr">
+        <is>
+          <t>MemberEthnicityCode1</t>
+        </is>
+      </c>
+      <c r="CE1" s="3" t="inlineStr">
+        <is>
+          <t>MemberEthnicityCode2</t>
+        </is>
+      </c>
+      <c r="CF1" s="3" t="inlineStr">
+        <is>
+          <t>MemberEthnicityCode3</t>
+        </is>
+      </c>
+      <c r="CG1" s="3" t="inlineStr">
         <is>
           <t>MemberCitizenshipCode</t>
         </is>
       </c>
-      <c r="CC1" s="3" t="inlineStr">
+      <c r="CH1" s="3" t="inlineStr">
         <is>
           <t>MemberEmploymentClassCode1</t>
         </is>
       </c>
-      <c r="CD1" s="3" t="inlineStr">
+      <c r="CI1" s="3" t="inlineStr">
         <is>
           <t>MemberEmploymentClassCode2</t>
         </is>
       </c>
-      <c r="CE1" s="3" t="inlineStr">
+      <c r="CJ1" s="3" t="inlineStr">
         <is>
           <t>MemberEmploymentClassCode3</t>
         </is>
       </c>
-      <c r="CF1" s="3" t="inlineStr">
+      <c r="CK1" s="3" t="inlineStr">
         <is>
           <t>MemberEmploymentClassCode4</t>
         </is>
       </c>
-      <c r="CG1" s="3" t="inlineStr">
+      <c r="CL1" s="3" t="inlineStr">
         <is>
           <t>MemberEmploymentClassCode5</t>
         </is>
       </c>
-      <c r="CH1" s="3" t="inlineStr">
+      <c r="CM1" s="3" t="inlineStr">
         <is>
           <t>MemberWageFrequencyCode</t>
         </is>
       </c>
-      <c r="CI1" s="3" t="inlineStr">
+      <c r="CN1" s="3" t="inlineStr">
         <is>
           <t>MemberWageAmount</t>
         </is>
       </c>
-      <c r="CJ1" s="3" t="inlineStr">
+      <c r="CO1" s="3" t="inlineStr">
         <is>
           <t>MemberWorkHoursCount</t>
         </is>
       </c>
-      <c r="CK1" s="3" t="inlineStr">
+      <c r="CP1" s="3" t="inlineStr">
         <is>
           <t>MemberEmployerLocationIdentificationCode</t>
         </is>
       </c>
-      <c r="CL1" s="3" t="inlineStr">
+      <c r="CQ1" s="3" t="inlineStr">
         <is>
           <t>MemberSalaryGradeCode</t>
         </is>
       </c>
-      <c r="CM1" s="3" t="inlineStr">
+      <c r="CR1" s="3" t="inlineStr">
         <is>
           <t>MemberHealthRelatedCode</t>
         </is>
       </c>
-      <c r="CN1" s="3" t="inlineStr">
+      <c r="CS1" s="3" t="inlineStr">
         <is>
           <t>MemberHeight</t>
         </is>
       </c>
-      <c r="CO1" s="3" t="inlineStr">
+      <c r="CT1" s="3" t="inlineStr">
         <is>
           <t>MemberWeight</t>
         </is>
       </c>
-      <c r="CP1" s="3" t="inlineStr">
+      <c r="CU1" s="3" t="inlineStr">
         <is>
           <t>MemberLanguageInfoCodeQualifier</t>
         </is>
       </c>
-      <c r="CQ1" s="3" t="inlineStr">
+      <c r="CV1" s="3" t="inlineStr">
         <is>
           <t>MemberLanguageInfoCode</t>
         </is>
       </c>
-      <c r="CR1" s="3" t="inlineStr">
+      <c r="CW1" s="3" t="inlineStr">
         <is>
           <t>MemberLanguageInfoLanguageDescription</t>
         </is>
       </c>
-      <c r="CS1" s="3" t="inlineStr">
+      <c r="CX1" s="3" t="inlineStr">
         <is>
           <t>MemberLanguageInfoLanguageUseIndicator</t>
         </is>
       </c>
-      <c r="CT1" s="3" t="inlineStr">
+      <c r="CY1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberIdentifier</t>
         </is>
       </c>
-      <c r="CU1" s="3" t="inlineStr">
+      <c r="CZ1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberLastName</t>
         </is>
       </c>
-      <c r="CV1" s="3" t="inlineStr">
+      <c r="DA1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberFirstName</t>
         </is>
       </c>
-      <c r="CW1" s="3" t="inlineStr">
+      <c r="DB1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberMiddleName</t>
         </is>
       </c>
-      <c r="CX1" s="3" t="inlineStr">
+      <c r="DC1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberBirthDate</t>
         </is>
       </c>
-      <c r="CY1" s="3" t="inlineStr">
+      <c r="DD1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberGender</t>
         </is>
       </c>
-      <c r="CZ1" s="3" t="inlineStr">
+      <c r="DE1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberMaritalStatusCode</t>
         </is>
       </c>
-      <c r="DA1" s="3" t="inlineStr">
+      <c r="DF1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberEthnicityCode</t>
         </is>
       </c>
-      <c r="DB1" s="3" t="inlineStr">
+      <c r="DG1" s="3" t="inlineStr">
         <is>
           <t>IncorrectMemberCitizenshipCode</t>
         </is>
       </c>
-      <c r="DC1" s="3" t="inlineStr">
+      <c r="DH1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount1QualifierCode</t>
         </is>
       </c>
-      <c r="DD1" s="3" t="inlineStr">
+      <c r="DI1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount1Amount</t>
         </is>
       </c>
-      <c r="DE1" s="3" t="inlineStr">
+      <c r="DJ1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount2QualifierCode</t>
         </is>
       </c>
-      <c r="DF1" s="3" t="inlineStr">
+      <c r="DK1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount2Amount</t>
         </is>
       </c>
-      <c r="DG1" s="3" t="inlineStr">
+      <c r="DL1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount3QualifierCode</t>
         </is>
       </c>
-      <c r="DH1" s="3" t="inlineStr">
+      <c r="DM1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount3Amount</t>
         </is>
       </c>
-      <c r="DI1" s="3" t="inlineStr">
+      <c r="DN1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount4QualifierCode</t>
         </is>
       </c>
-      <c r="DJ1" s="3" t="inlineStr">
+      <c r="DO1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount4Amount</t>
         </is>
       </c>
-      <c r="DK1" s="3" t="inlineStr">
+      <c r="DP1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount5QualifierCode</t>
         </is>
       </c>
-      <c r="DL1" s="3" t="inlineStr">
+      <c r="DQ1" s="3" t="inlineStr">
         <is>
           <t>ContractAmount5Amount</t>
         </is>
       </c>
-      <c r="DM1" s="3" t="inlineStr">
+      <c r="DR1" s="3" t="inlineStr">
         <is>
           <t>MailingAddressLine</t>
         </is>
       </c>
-      <c r="DN1" s="3" t="inlineStr">
+      <c r="DS1" s="3" t="inlineStr">
         <is>
           <t>MailingAddressLine2</t>
         </is>
       </c>
-      <c r="DO1" s="3" t="inlineStr">
+      <c r="DT1" s="3" t="inlineStr">
         <is>
           <t>MailingAddressCity</t>
         </is>
       </c>
-      <c r="DP1" s="3" t="inlineStr">
+      <c r="DU1" s="3" t="inlineStr">
         <is>
           <t>MailingAddressStateCode</t>
         </is>
       </c>
-      <c r="DQ1" s="3" t="inlineStr">
+      <c r="DV1" s="3" t="inlineStr">
         <is>
           <t>MailingAddressZipCode</t>
         </is>
       </c>
-      <c r="DR1" s="3" t="inlineStr">
+      <c r="DW1" s="3" t="inlineStr">
         <is>
           <t>Employer1Identifier</t>
         </is>
       </c>
-      <c r="DS1" s="3" t="inlineStr">
+      <c r="DX1" s="3" t="inlineStr">
         <is>
           <t>Employer1LastNameOrOrgName</t>
         </is>
       </c>
-      <c r="DT1" s="3" t="inlineStr">
+      <c r="DY1" s="3" t="inlineStr">
         <is>
           <t>Employer1FirstName</t>
         </is>
       </c>
-      <c r="DU1" s="3" t="inlineStr">
+      <c r="DZ1" s="3" t="inlineStr">
         <is>
           <t>Employer1MiddleName</t>
         </is>
       </c>
-      <c r="DV1" s="3" t="inlineStr">
+      <c r="EA1" s="3" t="inlineStr">
         <is>
           <t>Employer1AddressLine</t>
         </is>
       </c>
-      <c r="DW1" s="3" t="inlineStr">
+      <c r="EB1" s="3" t="inlineStr">
         <is>
           <t>Employer1AddressLine2</t>
         </is>
       </c>
-      <c r="DX1" s="3" t="inlineStr">
+      <c r="EC1" s="3" t="inlineStr">
         <is>
           <t>Employer1AddressCity</t>
         </is>
       </c>
-      <c r="DY1" s="3" t="inlineStr">
+      <c r="ED1" s="3" t="inlineStr">
         <is>
           <t>Employer1AddressStateCode</t>
         </is>
       </c>
-      <c r="DZ1" s="3" t="inlineStr">
+      <c r="EE1" s="3" t="inlineStr">
         <is>
           <t>Employer1AddressZipCode</t>
         </is>
       </c>
-      <c r="EA1" s="3" t="inlineStr">
+      <c r="EF1" s="3" t="inlineStr">
         <is>
           <t>Employer1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="EB1" s="3" t="inlineStr">
+      <c r="EG1" s="3" t="inlineStr">
         <is>
           <t>Employer1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="EC1" s="3" t="inlineStr">
+      <c r="EH1" s="3" t="inlineStr">
         <is>
           <t>Employer1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="ED1" s="3" t="inlineStr">
+      <c r="EI1" s="3" t="inlineStr">
         <is>
           <t>Employer1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="EE1" s="3" t="inlineStr">
+      <c r="EJ1" s="3" t="inlineStr">
         <is>
           <t>Employer2Identifier</t>
         </is>
       </c>
-      <c r="EF1" s="3" t="inlineStr">
+      <c r="EK1" s="3" t="inlineStr">
         <is>
           <t>Employer2LastNameOrOrgName</t>
         </is>
       </c>
-      <c r="EG1" s="3" t="inlineStr">
+      <c r="EL1" s="3" t="inlineStr">
         <is>
           <t>Employer2FirstName</t>
         </is>
       </c>
-      <c r="EH1" s="3" t="inlineStr">
+      <c r="EM1" s="3" t="inlineStr">
         <is>
           <t>Employer2MiddleName</t>
         </is>
       </c>
-      <c r="EI1" s="3" t="inlineStr">
+      <c r="EN1" s="3" t="inlineStr">
         <is>
           <t>Employer2AddressLine</t>
         </is>
       </c>
-      <c r="EJ1" s="3" t="inlineStr">
+      <c r="EO1" s="3" t="inlineStr">
         <is>
           <t>Employer2AddressLine2</t>
         </is>
       </c>
-      <c r="EK1" s="3" t="inlineStr">
+      <c r="EP1" s="3" t="inlineStr">
         <is>
           <t>Employer2AddressCity</t>
         </is>
       </c>
-      <c r="EL1" s="3" t="inlineStr">
+      <c r="EQ1" s="3" t="inlineStr">
         <is>
           <t>Employer2AddressStateCode</t>
         </is>
       </c>
-      <c r="EM1" s="3" t="inlineStr">
+      <c r="ER1" s="3" t="inlineStr">
         <is>
           <t>Employer2AddressZipCode</t>
         </is>
       </c>
-      <c r="EN1" s="3" t="inlineStr">
+      <c r="ES1" s="3" t="inlineStr">
         <is>
           <t>Employer2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="EO1" s="3" t="inlineStr">
+      <c r="ET1" s="3" t="inlineStr">
         <is>
           <t>Employer2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="EP1" s="3" t="inlineStr">
+      <c r="EU1" s="3" t="inlineStr">
         <is>
           <t>Employer2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="EQ1" s="3" t="inlineStr">
+      <c r="EV1" s="3" t="inlineStr">
         <is>
           <t>Employer2ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="ER1" s="3" t="inlineStr">
+      <c r="EW1" s="3" t="inlineStr">
         <is>
           <t>School1Identifier</t>
         </is>
       </c>
-      <c r="ES1" s="3" t="inlineStr">
+      <c r="EX1" s="3" t="inlineStr">
         <is>
           <t>School1Name</t>
         </is>
       </c>
-      <c r="ET1" s="3" t="inlineStr">
+      <c r="EY1" s="3" t="inlineStr">
         <is>
           <t>School1AddressLine</t>
         </is>
       </c>
-      <c r="EU1" s="3" t="inlineStr">
+      <c r="EZ1" s="3" t="inlineStr">
         <is>
           <t>School1AddressLine2</t>
         </is>
       </c>
-      <c r="EV1" s="3" t="inlineStr">
+      <c r="FA1" s="3" t="inlineStr">
         <is>
           <t>School1AddressCity</t>
         </is>
       </c>
-      <c r="EW1" s="3" t="inlineStr">
+      <c r="FB1" s="3" t="inlineStr">
         <is>
           <t>School1AddressStateCode</t>
         </is>
       </c>
-      <c r="EX1" s="3" t="inlineStr">
+      <c r="FC1" s="3" t="inlineStr">
         <is>
           <t>School1AddressZipCode</t>
         </is>
       </c>
-      <c r="EY1" s="3" t="inlineStr">
+      <c r="FD1" s="3" t="inlineStr">
         <is>
           <t>School1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="EZ1" s="3" t="inlineStr">
+      <c r="FE1" s="3" t="inlineStr">
         <is>
           <t>School1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="FA1" s="3" t="inlineStr">
+      <c r="FF1" s="3" t="inlineStr">
         <is>
           <t>School1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="FB1" s="3" t="inlineStr">
+      <c r="FG1" s="3" t="inlineStr">
         <is>
           <t>School1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="FC1" s="3" t="inlineStr">
+      <c r="FH1" s="3" t="inlineStr">
         <is>
           <t>School2Identifier</t>
         </is>
       </c>
-      <c r="FD1" s="3" t="inlineStr">
+      <c r="FI1" s="3" t="inlineStr">
         <is>
           <t>School2Name</t>
         </is>
       </c>
-      <c r="FE1" s="3" t="inlineStr">
+      <c r="FJ1" s="3" t="inlineStr">
         <is>
           <t>School2AddressLine</t>
         </is>
       </c>
-      <c r="FF1" s="3" t="inlineStr">
+      <c r="FK1" s="3" t="inlineStr">
         <is>
           <t>School2AddressLine2</t>
         </is>
       </c>
-      <c r="FG1" s="3" t="inlineStr">
+      <c r="FL1" s="3" t="inlineStr">
         <is>
           <t>School2AddressCity</t>
         </is>
       </c>
-      <c r="FH1" s="3" t="inlineStr">
+      <c r="FM1" s="3" t="inlineStr">
         <is>
           <t>School2AddressStateCode</t>
         </is>
       </c>
-      <c r="FI1" s="3" t="inlineStr">
+      <c r="FN1" s="3" t="inlineStr">
         <is>
           <t>School2AddressZipCode</t>
         </is>
       </c>
-      <c r="FJ1" s="3" t="inlineStr">
+      <c r="FO1" s="3" t="inlineStr">
         <is>
           <t>School2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="FK1" s="3" t="inlineStr">
+      <c r="FP1" s="3" t="inlineStr">
         <is>
           <t>School2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="FL1" s="3" t="inlineStr">
+      <c r="FQ1" s="3" t="inlineStr">
         <is>
           <t>School2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="FM1" s="3" t="inlineStr">
+      <c r="FR1" s="3" t="inlineStr">
         <is>
           <t>School2ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="FN1" s="3" t="inlineStr">
+      <c r="FS1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentIdentifier</t>
         </is>
       </c>
-      <c r="FO1" s="3" t="inlineStr">
+      <c r="FT1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentLastName</t>
         </is>
       </c>
-      <c r="FP1" s="3" t="inlineStr">
+      <c r="FU1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentFirstName</t>
         </is>
       </c>
-      <c r="FQ1" s="3" t="inlineStr">
+      <c r="FV1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentMiddleName</t>
         </is>
       </c>
-      <c r="FR1" s="3" t="inlineStr">
+      <c r="FW1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentAddressLine</t>
         </is>
       </c>
-      <c r="FS1" s="3" t="inlineStr">
+      <c r="FX1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentAddressLine2</t>
         </is>
       </c>
-      <c r="FT1" s="3" t="inlineStr">
+      <c r="FY1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentAddressCity</t>
         </is>
       </c>
-      <c r="FU1" s="3" t="inlineStr">
+      <c r="FZ1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentAddressStateCode</t>
         </is>
       </c>
-      <c r="FV1" s="3" t="inlineStr">
+      <c r="GA1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentAddressZipCode</t>
         </is>
       </c>
-      <c r="FW1" s="3" t="inlineStr">
+      <c r="GB1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="FX1" s="3" t="inlineStr">
+      <c r="GC1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="FY1" s="3" t="inlineStr">
+      <c r="GD1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="FZ1" s="3" t="inlineStr">
+      <c r="GE1" s="3" t="inlineStr">
         <is>
           <t>CustodialParentContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="GA1" s="3" t="inlineStr">
+      <c r="GF1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1EntityRole</t>
         </is>
       </c>
-      <c r="GB1" s="3" t="inlineStr">
+      <c r="GG1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1Identifier</t>
         </is>
       </c>
-      <c r="GC1" s="3" t="inlineStr">
+      <c r="GH1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1LastName</t>
         </is>
       </c>
-      <c r="GD1" s="3" t="inlineStr">
+      <c r="GI1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1FirstName</t>
         </is>
       </c>
-      <c r="GE1" s="3" t="inlineStr">
+      <c r="GJ1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1MiddleName</t>
         </is>
       </c>
-      <c r="GF1" s="3" t="inlineStr">
+      <c r="GK1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1AddressLine</t>
         </is>
       </c>
-      <c r="GG1" s="3" t="inlineStr">
+      <c r="GL1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1AddressLine2</t>
         </is>
       </c>
-      <c r="GH1" s="3" t="inlineStr">
+      <c r="GM1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1AddressCity</t>
         </is>
       </c>
-      <c r="GI1" s="3" t="inlineStr">
+      <c r="GN1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1AddressStateCode</t>
         </is>
       </c>
-      <c r="GJ1" s="3" t="inlineStr">
+      <c r="GO1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1AddressZipCode</t>
         </is>
       </c>
-      <c r="GK1" s="3" t="inlineStr">
+      <c r="GP1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="GL1" s="3" t="inlineStr">
+      <c r="GQ1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="GM1" s="3" t="inlineStr">
+      <c r="GR1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="GN1" s="3" t="inlineStr">
+      <c r="GS1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="GO1" s="3" t="inlineStr">
+      <c r="GT1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2EntityRole</t>
         </is>
       </c>
-      <c r="GP1" s="3" t="inlineStr">
+      <c r="GU1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2Identifier</t>
         </is>
       </c>
-      <c r="GQ1" s="3" t="inlineStr">
+      <c r="GV1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2LastName</t>
         </is>
       </c>
-      <c r="GR1" s="3" t="inlineStr">
+      <c r="GW1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2FirstName</t>
         </is>
       </c>
-      <c r="GS1" s="3" t="inlineStr">
+      <c r="GX1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2MiddleName</t>
         </is>
       </c>
-      <c r="GT1" s="3" t="inlineStr">
+      <c r="GY1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2AddressLine</t>
         </is>
       </c>
-      <c r="GU1" s="3" t="inlineStr">
+      <c r="GZ1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2AddressLine2</t>
         </is>
       </c>
-      <c r="GV1" s="3" t="inlineStr">
+      <c r="HA1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2AddressCity</t>
         </is>
       </c>
-      <c r="GW1" s="3" t="inlineStr">
+      <c r="HB1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2AddressStateCode</t>
         </is>
       </c>
-      <c r="GX1" s="3" t="inlineStr">
+      <c r="HC1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2AddressZipCode</t>
         </is>
       </c>
-      <c r="GY1" s="3" t="inlineStr">
+      <c r="HD1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="GZ1" s="3" t="inlineStr">
+      <c r="HE1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="HA1" s="3" t="inlineStr">
+      <c r="HF1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="HB1" s="3" t="inlineStr">
+      <c r="HG1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson2ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="HC1" s="3" t="inlineStr">
+      <c r="HH1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3EntityRole</t>
         </is>
       </c>
-      <c r="HD1" s="3" t="inlineStr">
+      <c r="HI1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3Identifier</t>
         </is>
       </c>
-      <c r="HE1" s="3" t="inlineStr">
+      <c r="HJ1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3LastName</t>
         </is>
       </c>
-      <c r="HF1" s="3" t="inlineStr">
+      <c r="HK1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3FirstName</t>
         </is>
       </c>
-      <c r="HG1" s="3" t="inlineStr">
+      <c r="HL1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3MiddleName</t>
         </is>
       </c>
-      <c r="HH1" s="3" t="inlineStr">
+      <c r="HM1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3AddressLine</t>
         </is>
       </c>
-      <c r="HI1" s="3" t="inlineStr">
+      <c r="HN1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3AddressLine2</t>
         </is>
       </c>
-      <c r="HJ1" s="3" t="inlineStr">
+      <c r="HO1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3AddressCity</t>
         </is>
       </c>
-      <c r="HK1" s="3" t="inlineStr">
+      <c r="HP1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3AddressStateCode</t>
         </is>
       </c>
-      <c r="HL1" s="3" t="inlineStr">
+      <c r="HQ1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3AddressZipCode</t>
         </is>
       </c>
-      <c r="HM1" s="3" t="inlineStr">
+      <c r="HR1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="HN1" s="3" t="inlineStr">
+      <c r="HS1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="HO1" s="3" t="inlineStr">
+      <c r="HT1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="HP1" s="3" t="inlineStr">
+      <c r="HU1" s="3" t="inlineStr">
         <is>
           <t>ResponsiblePerson3ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="HQ1" s="3" t="inlineStr">
+      <c r="HV1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationLastNameOrOrgName</t>
         </is>
       </c>
-      <c r="HR1" s="3" t="inlineStr">
+      <c r="HW1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationFirstName</t>
         </is>
       </c>
-      <c r="HS1" s="3" t="inlineStr">
+      <c r="HX1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationMiddleName</t>
         </is>
       </c>
-      <c r="HT1" s="3" t="inlineStr">
+      <c r="HY1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationAddressLine</t>
         </is>
       </c>
-      <c r="HU1" s="3" t="inlineStr">
+      <c r="HZ1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationAddressLine2</t>
         </is>
       </c>
-      <c r="HV1" s="3" t="inlineStr">
+      <c r="IA1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationAddressCity</t>
         </is>
       </c>
-      <c r="HW1" s="3" t="inlineStr">
+      <c r="IB1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationAddressStateCode</t>
         </is>
       </c>
-      <c r="HX1" s="3" t="inlineStr">
+      <c r="IC1" s="3" t="inlineStr">
         <is>
           <t>DropOffLocationAddressZipCode</t>
         </is>
       </c>
-      <c r="HY1" s="3" t="inlineStr">
+      <c r="ID1" s="3" t="inlineStr">
         <is>
           <t>Disability1TypeCode</t>
         </is>
       </c>
-      <c r="HZ1" s="3" t="inlineStr">
+      <c r="IE1" s="3" t="inlineStr">
         <is>
           <t>Disability1DiagnosisCode</t>
         </is>
       </c>
-      <c r="IA1" s="3" t="inlineStr">
+      <c r="IF1" s="3" t="inlineStr">
         <is>
           <t>Disability1DateFrom</t>
         </is>
       </c>
-      <c r="IB1" s="3" t="inlineStr">
+      <c r="IG1" s="3" t="inlineStr">
         <is>
           <t>Disability1DateTo</t>
         </is>
       </c>
-      <c r="IC1" s="3" t="inlineStr">
+      <c r="IH1" s="3" t="inlineStr">
         <is>
           <t>Disability2TypeCode</t>
         </is>
       </c>
-      <c r="ID1" s="3" t="inlineStr">
+      <c r="II1" s="3" t="inlineStr">
         <is>
           <t>Disability2DiagnosisCode</t>
         </is>
       </c>
-      <c r="IE1" s="3" t="inlineStr">
+      <c r="IJ1" s="3" t="inlineStr">
         <is>
           <t>Disability2DateFrom</t>
         </is>
       </c>
-      <c r="IF1" s="3" t="inlineStr">
+      <c r="IK1" s="3" t="inlineStr">
         <is>
           <t>Disability2DateTo</t>
         </is>
       </c>
-      <c r="IG1" s="3" t="inlineStr">
+      <c r="IL1" s="3" t="inlineStr">
         <is>
           <t>Disability3TypeCode</t>
         </is>
       </c>
-      <c r="IH1" s="3" t="inlineStr">
+      <c r="IM1" s="3" t="inlineStr">
         <is>
           <t>Disability3DiagnosisCode</t>
         </is>
       </c>
-      <c r="II1" s="3" t="inlineStr">
+      <c r="IN1" s="3" t="inlineStr">
         <is>
           <t>Disability3DateFrom</t>
         </is>
       </c>
-      <c r="IJ1" s="3" t="inlineStr">
+      <c r="IO1" s="3" t="inlineStr">
         <is>
           <t>Disability3DateTo</t>
         </is>
       </c>
-      <c r="IK1" s="3" t="inlineStr">
+      <c r="IP1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1Name</t>
         </is>
       </c>
-      <c r="IL1" s="3" t="inlineStr">
+      <c r="IQ1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1IdentifierQualifierCode</t>
         </is>
       </c>
-      <c r="IM1" s="3" t="inlineStr">
+      <c r="IR1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1IdentifierType</t>
         </is>
       </c>
-      <c r="IN1" s="3" t="inlineStr">
+      <c r="IS1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1Identifier</t>
         </is>
       </c>
-      <c r="IO1" s="3" t="inlineStr">
+      <c r="IT1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1Date</t>
         </is>
       </c>
-      <c r="IP1" s="3" t="inlineStr">
+      <c r="IU1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory1DateTo</t>
         </is>
       </c>
-      <c r="IQ1" s="3" t="inlineStr">
+      <c r="IV1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2Name</t>
         </is>
       </c>
-      <c r="IR1" s="3" t="inlineStr">
+      <c r="IW1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2IdentifierQualifierCode</t>
         </is>
       </c>
-      <c r="IS1" s="3" t="inlineStr">
+      <c r="IX1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2IdentifierType</t>
         </is>
       </c>
-      <c r="IT1" s="3" t="inlineStr">
+      <c r="IY1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2Identifier</t>
         </is>
       </c>
-      <c r="IU1" s="3" t="inlineStr">
+      <c r="IZ1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2Date</t>
         </is>
       </c>
-      <c r="IV1" s="3" t="inlineStr">
+      <c r="JA1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory2DateTo</t>
         </is>
       </c>
-      <c r="IW1" s="3" t="inlineStr">
+      <c r="JB1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3Name</t>
         </is>
       </c>
-      <c r="IX1" s="3" t="inlineStr">
+      <c r="JC1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3IdentifierQualifierCode</t>
         </is>
       </c>
-      <c r="IY1" s="3" t="inlineStr">
+      <c r="JD1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3IdentifierType</t>
         </is>
       </c>
-      <c r="IZ1" s="3" t="inlineStr">
+      <c r="JE1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3Identifier</t>
         </is>
       </c>
-      <c r="JA1" s="3" t="inlineStr">
+      <c r="JF1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3Date</t>
         </is>
       </c>
-      <c r="JB1" s="3" t="inlineStr">
+      <c r="JG1" s="3" t="inlineStr">
         <is>
           <t>ReportingCategory3DateTo</t>
         </is>
       </c>
-      <c r="JC1" s="3" t="inlineStr">
+      <c r="JH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageMaintenanceTypeCode</t>
         </is>
       </c>
-      <c r="JD1" s="3" t="inlineStr">
+      <c r="JI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageInsuranceLineCode</t>
         </is>
       </c>
-      <c r="JE1" s="3" t="inlineStr">
+      <c r="JJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoveragePlanDescription</t>
         </is>
       </c>
-      <c r="JF1" s="3" t="inlineStr">
+      <c r="JK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageLevelCode</t>
         </is>
       </c>
-      <c r="JG1" s="3" t="inlineStr">
+      <c r="JL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageLateEnrollmentIndicator</t>
         </is>
       </c>
-      <c r="JH1" s="3" t="inlineStr">
+      <c r="JM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate1QualifierCode</t>
         </is>
       </c>
-      <c r="JI1" s="3" t="inlineStr">
+      <c r="JN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate1Date</t>
         </is>
       </c>
-      <c r="JJ1" s="3" t="inlineStr">
+      <c r="JO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate2QualifierCode</t>
         </is>
       </c>
-      <c r="JK1" s="3" t="inlineStr">
+      <c r="JP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate2Date</t>
         </is>
       </c>
-      <c r="JL1" s="3" t="inlineStr">
+      <c r="JQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate3QualifierCode</t>
         </is>
       </c>
-      <c r="JM1" s="3" t="inlineStr">
+      <c r="JR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate3Date</t>
         </is>
       </c>
-      <c r="JN1" s="3" t="inlineStr">
+      <c r="JS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate4QualifierCode</t>
         </is>
       </c>
-      <c r="JO1" s="3" t="inlineStr">
+      <c r="JT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate4Date</t>
         </is>
       </c>
-      <c r="JP1" s="3" t="inlineStr">
+      <c r="JU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate5QualifierCode</t>
         </is>
       </c>
-      <c r="JQ1" s="3" t="inlineStr">
+      <c r="JV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCoverageDate5Date</t>
         </is>
       </c>
-      <c r="JR1" s="3" t="inlineStr">
+      <c r="JW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount1QualifierCode</t>
         </is>
       </c>
-      <c r="JS1" s="3" t="inlineStr">
+      <c r="JX1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount1Amount</t>
         </is>
       </c>
-      <c r="JT1" s="3" t="inlineStr">
+      <c r="JY1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount2QualifierCode</t>
         </is>
       </c>
-      <c r="JU1" s="3" t="inlineStr">
+      <c r="JZ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount2Amount</t>
         </is>
       </c>
-      <c r="JV1" s="3" t="inlineStr">
+      <c r="KA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount3QualifierCode</t>
         </is>
       </c>
-      <c r="JW1" s="3" t="inlineStr">
+      <c r="KB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageContractAmount3Amount</t>
         </is>
       </c>
-      <c r="JX1" s="3" t="inlineStr">
+      <c r="KC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber1QualifierCode</t>
         </is>
       </c>
-      <c r="JY1" s="3" t="inlineStr">
+      <c r="KD1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber1Identification</t>
         </is>
       </c>
-      <c r="JZ1" s="3" t="inlineStr">
+      <c r="KE1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber2QualifierCode</t>
         </is>
       </c>
-      <c r="KA1" s="3" t="inlineStr">
+      <c r="KF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber2Identification</t>
         </is>
       </c>
-      <c r="KB1" s="3" t="inlineStr">
+      <c r="KG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber3QualifierCode</t>
         </is>
       </c>
-      <c r="KC1" s="3" t="inlineStr">
+      <c r="KH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber3Identification</t>
         </is>
       </c>
-      <c r="KD1" s="3" t="inlineStr">
+      <c r="KI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber4QualifierCode</t>
         </is>
       </c>
-      <c r="KE1" s="3" t="inlineStr">
+      <c r="KJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber4Identification</t>
         </is>
       </c>
-      <c r="KF1" s="3" t="inlineStr">
+      <c r="KK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber5QualifierCode</t>
         </is>
       </c>
-      <c r="KG1" s="3" t="inlineStr">
+      <c r="KL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageGroupOrPolicyNumber5Identification</t>
         </is>
       </c>
-      <c r="KH1" s="3" t="inlineStr">
+      <c r="KM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoveragePriorCoverageMonthCount</t>
         </is>
       </c>
-      <c r="KI1" s="3" t="inlineStr">
+      <c r="KN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageIdCardPlanDesc</t>
         </is>
       </c>
-      <c r="KJ1" s="3" t="inlineStr">
+      <c r="KO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageIdCardTypeCode</t>
         </is>
       </c>
-      <c r="KK1" s="3" t="inlineStr">
+      <c r="KP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageIdCardCount</t>
         </is>
       </c>
-      <c r="KL1" s="3" t="inlineStr">
+      <c r="KQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageIdCardActionCode</t>
         </is>
       </c>
-      <c r="KM1" s="3" t="inlineStr">
+      <c r="KR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1EntityRole</t>
         </is>
       </c>
-      <c r="KN1" s="3" t="inlineStr">
+      <c r="KS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1EntityType</t>
         </is>
       </c>
-      <c r="KO1" s="3" t="inlineStr">
+      <c r="KT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1Identifier</t>
         </is>
       </c>
-      <c r="KP1" s="3" t="inlineStr">
+      <c r="KU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1LastNameOrOrgName</t>
         </is>
       </c>
-      <c r="KQ1" s="3" t="inlineStr">
+      <c r="KV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1FirstName</t>
         </is>
       </c>
-      <c r="KR1" s="3" t="inlineStr">
+      <c r="KW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1MiddleName</t>
         </is>
       </c>
-      <c r="KS1" s="3" t="inlineStr">
+      <c r="KX1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1AddressLine</t>
         </is>
       </c>
-      <c r="KT1" s="3" t="inlineStr">
+      <c r="KY1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1AddressLine2</t>
         </is>
       </c>
-      <c r="KU1" s="3" t="inlineStr">
+      <c r="KZ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1AddressCity</t>
         </is>
       </c>
-      <c r="KV1" s="3" t="inlineStr">
+      <c r="LA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1AddressStateCode</t>
         </is>
       </c>
-      <c r="KW1" s="3" t="inlineStr">
+      <c r="LB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1AddressZipCode</t>
         </is>
       </c>
-      <c r="KX1" s="3" t="inlineStr">
+      <c r="LC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="KY1" s="3" t="inlineStr">
+      <c r="LD1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="KZ1" s="3" t="inlineStr">
+      <c r="LE1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="LA1" s="3" t="inlineStr">
+      <c r="LF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="LB1" s="3" t="inlineStr">
+      <c r="LG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ChangeReasonActionCode</t>
         </is>
       </c>
-      <c r="LC1" s="3" t="inlineStr">
+      <c r="LH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ChangeReasonEffectiveDate</t>
         </is>
       </c>
-      <c r="LD1" s="3" t="inlineStr">
+      <c r="LI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider1ChangeReasonReasonCode</t>
         </is>
       </c>
-      <c r="LE1" s="3" t="inlineStr">
+      <c r="LJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2EntityRole</t>
         </is>
       </c>
-      <c r="LF1" s="3" t="inlineStr">
+      <c r="LK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2EntityType</t>
         </is>
       </c>
-      <c r="LG1" s="3" t="inlineStr">
+      <c r="LL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2Identifier</t>
         </is>
       </c>
-      <c r="LH1" s="3" t="inlineStr">
+      <c r="LM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2LastNameOrOrgName</t>
         </is>
       </c>
-      <c r="LI1" s="3" t="inlineStr">
+      <c r="LN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2FirstName</t>
         </is>
       </c>
-      <c r="LJ1" s="3" t="inlineStr">
+      <c r="LO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2MiddleName</t>
         </is>
       </c>
-      <c r="LK1" s="3" t="inlineStr">
+      <c r="LP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2AddressLine</t>
         </is>
       </c>
-      <c r="LL1" s="3" t="inlineStr">
+      <c r="LQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2AddressLine2</t>
         </is>
       </c>
-      <c r="LM1" s="3" t="inlineStr">
+      <c r="LR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2AddressCity</t>
         </is>
       </c>
-      <c r="LN1" s="3" t="inlineStr">
+      <c r="LS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2AddressStateCode</t>
         </is>
       </c>
-      <c r="LO1" s="3" t="inlineStr">
+      <c r="LT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2AddressZipCode</t>
         </is>
       </c>
-      <c r="LP1" s="3" t="inlineStr">
+      <c r="LU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="LQ1" s="3" t="inlineStr">
+      <c r="LV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="LR1" s="3" t="inlineStr">
+      <c r="LW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="LS1" s="3" t="inlineStr">
+      <c r="LX1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="LT1" s="3" t="inlineStr">
+      <c r="LY1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ChangeReasonActionCode</t>
         </is>
       </c>
-      <c r="LU1" s="3" t="inlineStr">
+      <c r="LZ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ChangeReasonEffectiveDate</t>
         </is>
       </c>
-      <c r="LV1" s="3" t="inlineStr">
+      <c r="MA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider2ChangeReasonReasonCode</t>
         </is>
       </c>
-      <c r="LW1" s="3" t="inlineStr">
+      <c r="MB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3EntityRole</t>
         </is>
       </c>
-      <c r="LX1" s="3" t="inlineStr">
+      <c r="MC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3EntityType</t>
         </is>
       </c>
-      <c r="LY1" s="3" t="inlineStr">
+      <c r="MD1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3Identifier</t>
         </is>
       </c>
-      <c r="LZ1" s="3" t="inlineStr">
+      <c r="ME1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3LastNameOrOrgName</t>
         </is>
       </c>
-      <c r="MA1" s="3" t="inlineStr">
+      <c r="MF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3FirstName</t>
         </is>
       </c>
-      <c r="MB1" s="3" t="inlineStr">
+      <c r="MG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3MiddleName</t>
         </is>
       </c>
-      <c r="MC1" s="3" t="inlineStr">
+      <c r="MH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3AddressLine</t>
         </is>
       </c>
-      <c r="MD1" s="3" t="inlineStr">
+      <c r="MI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3AddressLine2</t>
         </is>
       </c>
-      <c r="ME1" s="3" t="inlineStr">
+      <c r="MJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3AddressCity</t>
         </is>
       </c>
-      <c r="MF1" s="3" t="inlineStr">
+      <c r="MK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3AddressStateCode</t>
         </is>
       </c>
-      <c r="MG1" s="3" t="inlineStr">
+      <c r="ML1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3AddressZipCode</t>
         </is>
       </c>
-      <c r="MH1" s="3" t="inlineStr">
+      <c r="MM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="MI1" s="3" t="inlineStr">
+      <c r="MN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="MJ1" s="3" t="inlineStr">
+      <c r="MO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="MK1" s="3" t="inlineStr">
+      <c r="MP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="ML1" s="3" t="inlineStr">
+      <c r="MQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ChangeReasonActionCode</t>
         </is>
       </c>
-      <c r="MM1" s="3" t="inlineStr">
+      <c r="MR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ChangeReasonEffectiveDate</t>
         </is>
       </c>
-      <c r="MN1" s="3" t="inlineStr">
+      <c r="MS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageProvider3ChangeReasonReasonCode</t>
         </is>
       </c>
-      <c r="MO1" s="3" t="inlineStr">
+      <c r="MT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1PayerResponsibilitySequenceCode</t>
         </is>
       </c>
-      <c r="MP1" s="3" t="inlineStr">
+      <c r="MU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1PayerResponsibilitySequence</t>
         </is>
       </c>
-      <c r="MQ1" s="3" t="inlineStr">
+      <c r="MV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1GroupOrPolicyNumber</t>
         </is>
       </c>
-      <c r="MR1" s="3" t="inlineStr">
+      <c r="MW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1CoordinationOfBenefitsCode</t>
         </is>
       </c>
-      <c r="MS1" s="3" t="inlineStr">
+      <c r="MX1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob1ServiceTypeCode1</t>
+        </is>
+      </c>
+      <c r="MY1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob1ServiceTypeCode2</t>
+        </is>
+      </c>
+      <c r="MZ1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob1ServiceTypeCode3</t>
+        </is>
+      </c>
+      <c r="NA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1AdditionalIdentifier1QualifierCode</t>
         </is>
       </c>
-      <c r="MT1" s="3" t="inlineStr">
+      <c r="NB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1AdditionalIdentifier1Identification</t>
         </is>
       </c>
-      <c r="MU1" s="3" t="inlineStr">
+      <c r="NC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1AdditionalIdentifier2QualifierCode</t>
         </is>
       </c>
-      <c r="MV1" s="3" t="inlineStr">
+      <c r="ND1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1AdditionalIdentifier2Identification</t>
         </is>
       </c>
-      <c r="MW1" s="3" t="inlineStr">
+      <c r="NE1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1DateFrom</t>
         </is>
       </c>
-      <c r="MX1" s="3" t="inlineStr">
+      <c r="NF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1DateTo</t>
         </is>
       </c>
-      <c r="MY1" s="3" t="inlineStr">
+      <c r="NG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1EntityRole</t>
         </is>
       </c>
-      <c r="MZ1" s="3" t="inlineStr">
+      <c r="NH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1Identifier</t>
         </is>
       </c>
-      <c r="NA1" s="3" t="inlineStr">
+      <c r="NI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1Name</t>
         </is>
       </c>
-      <c r="NB1" s="3" t="inlineStr">
+      <c r="NJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1AddressLine</t>
         </is>
       </c>
-      <c r="NC1" s="3" t="inlineStr">
+      <c r="NK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1AddressLine2</t>
         </is>
       </c>
-      <c r="ND1" s="3" t="inlineStr">
+      <c r="NL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1AddressCity</t>
         </is>
       </c>
-      <c r="NE1" s="3" t="inlineStr">
+      <c r="NM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1AddressStateCode</t>
         </is>
       </c>
-      <c r="NF1" s="3" t="inlineStr">
+      <c r="NN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1AddressZipCode</t>
         </is>
       </c>
-      <c r="NG1" s="3" t="inlineStr">
+      <c r="NO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="NH1" s="3" t="inlineStr">
+      <c r="NP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="NI1" s="3" t="inlineStr">
+      <c r="NQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="NJ1" s="3" t="inlineStr">
+      <c r="NR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="NK1" s="3" t="inlineStr">
+      <c r="NS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2EntityRole</t>
         </is>
       </c>
-      <c r="NL1" s="3" t="inlineStr">
+      <c r="NT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2Identifier</t>
         </is>
       </c>
-      <c r="NM1" s="3" t="inlineStr">
+      <c r="NU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2Name</t>
         </is>
       </c>
-      <c r="NN1" s="3" t="inlineStr">
+      <c r="NV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2AddressLine</t>
         </is>
       </c>
-      <c r="NO1" s="3" t="inlineStr">
+      <c r="NW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2AddressLine2</t>
         </is>
       </c>
-      <c r="NP1" s="3" t="inlineStr">
+      <c r="NX1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2AddressCity</t>
         </is>
       </c>
-      <c r="NQ1" s="3" t="inlineStr">
+      <c r="NY1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2AddressStateCode</t>
         </is>
       </c>
-      <c r="NR1" s="3" t="inlineStr">
+      <c r="NZ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2AddressZipCode</t>
         </is>
       </c>
-      <c r="NS1" s="3" t="inlineStr">
+      <c r="OA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="NT1" s="3" t="inlineStr">
+      <c r="OB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="NU1" s="3" t="inlineStr">
+      <c r="OC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="NV1" s="3" t="inlineStr">
+      <c r="OD1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob1Insurer2ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="NW1" s="3" t="inlineStr">
+      <c r="OE1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2PayerResponsibilitySequenceCode</t>
         </is>
       </c>
-      <c r="NX1" s="3" t="inlineStr">
+      <c r="OF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2PayerResponsibilitySequence</t>
         </is>
       </c>
-      <c r="NY1" s="3" t="inlineStr">
+      <c r="OG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2GroupOrPolicyNumber</t>
         </is>
       </c>
-      <c r="NZ1" s="3" t="inlineStr">
+      <c r="OH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2CoordinationOfBenefitsCode</t>
         </is>
       </c>
-      <c r="OA1" s="3" t="inlineStr">
+      <c r="OI1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob2ServiceTypeCode1</t>
+        </is>
+      </c>
+      <c r="OJ1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob2ServiceTypeCode2</t>
+        </is>
+      </c>
+      <c r="OK1" s="3" t="inlineStr">
+        <is>
+          <t>HealthCoverageCob2ServiceTypeCode3</t>
+        </is>
+      </c>
+      <c r="OL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2AdditionalIdentifier1QualifierCode</t>
         </is>
       </c>
-      <c r="OB1" s="3" t="inlineStr">
+      <c r="OM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2AdditionalIdentifier1Identification</t>
         </is>
       </c>
-      <c r="OC1" s="3" t="inlineStr">
+      <c r="ON1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2AdditionalIdentifier2QualifierCode</t>
         </is>
       </c>
-      <c r="OD1" s="3" t="inlineStr">
+      <c r="OO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2AdditionalIdentifier2Identification</t>
         </is>
       </c>
-      <c r="OE1" s="3" t="inlineStr">
+      <c r="OP1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2DateFrom</t>
         </is>
       </c>
-      <c r="OF1" s="3" t="inlineStr">
+      <c r="OQ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2DateTo</t>
         </is>
       </c>
-      <c r="OG1" s="3" t="inlineStr">
+      <c r="OR1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1EntityRole</t>
         </is>
       </c>
-      <c r="OH1" s="3" t="inlineStr">
+      <c r="OS1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1Identifier</t>
         </is>
       </c>
-      <c r="OI1" s="3" t="inlineStr">
+      <c r="OT1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1Name</t>
         </is>
       </c>
-      <c r="OJ1" s="3" t="inlineStr">
+      <c r="OU1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1AddressLine</t>
         </is>
       </c>
-      <c r="OK1" s="3" t="inlineStr">
+      <c r="OV1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1AddressLine2</t>
         </is>
       </c>
-      <c r="OL1" s="3" t="inlineStr">
+      <c r="OW1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1AddressCity</t>
         </is>
       </c>
-      <c r="OM1" s="3" t="inlineStr">
+      <c r="OX1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1AddressStateCode</t>
         </is>
       </c>
-      <c r="ON1" s="3" t="inlineStr">
+      <c r="OY1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1AddressZipCode</t>
         </is>
       </c>
-      <c r="OO1" s="3" t="inlineStr">
+      <c r="OZ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="OP1" s="3" t="inlineStr">
+      <c r="PA1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="OQ1" s="3" t="inlineStr">
+      <c r="PB1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="OR1" s="3" t="inlineStr">
+      <c r="PC1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer1ContactContactNumber2Number</t>
         </is>
       </c>
-      <c r="OS1" s="3" t="inlineStr">
+      <c r="PD1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2EntityRole</t>
         </is>
       </c>
-      <c r="OT1" s="3" t="inlineStr">
+      <c r="PE1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2Identifier</t>
         </is>
       </c>
-      <c r="OU1" s="3" t="inlineStr">
+      <c r="PF1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2Name</t>
         </is>
       </c>
-      <c r="OV1" s="3" t="inlineStr">
+      <c r="PG1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2AddressLine</t>
         </is>
       </c>
-      <c r="OW1" s="3" t="inlineStr">
+      <c r="PH1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2AddressLine2</t>
         </is>
       </c>
-      <c r="OX1" s="3" t="inlineStr">
+      <c r="PI1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2AddressCity</t>
         </is>
       </c>
-      <c r="OY1" s="3" t="inlineStr">
+      <c r="PJ1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2AddressStateCode</t>
         </is>
       </c>
-      <c r="OZ1" s="3" t="inlineStr">
+      <c r="PK1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2AddressZipCode</t>
         </is>
       </c>
-      <c r="PA1" s="3" t="inlineStr">
+      <c r="PL1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2ContactContactNumber1Type</t>
         </is>
       </c>
-      <c r="PB1" s="3" t="inlineStr">
+      <c r="PM1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2ContactContactNumber1Number</t>
         </is>
       </c>
-      <c r="PC1" s="3" t="inlineStr">
+      <c r="PN1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2ContactContactNumber2Type</t>
         </is>
       </c>
-      <c r="PD1" s="3" t="inlineStr">
+      <c r="PO1" s="3" t="inlineStr">
         <is>
           <t>HealthCoverageCob2Insurer2ContactContactNumber2Number</t>
         </is>
@@ -2167,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>690141ec7c0fb18b049a032c</t>
+          <t>6976904ee9a75feb6485564a</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2258,27 +2313,27 @@
       </c>
       <c r="AF2"/>
       <c r="AG2"/>
-      <c r="AH2" s="3" t="inlineStr">
+      <c r="AH2"/>
+      <c r="AI2"/>
+      <c r="AJ2" s="3" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="AI2"/>
-      <c r="AJ2"/>
       <c r="AK2"/>
-      <c r="AL2" s="3" t="inlineStr">
+      <c r="AL2"/>
+      <c r="AM2"/>
+      <c r="AN2"/>
+      <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>123456789</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AP2" s="3" t="inlineStr">
         <is>
           <t>123456001</t>
         </is>
       </c>
-      <c r="AN2"/>
-      <c r="AO2"/>
-      <c r="AP2"/>
       <c r="AQ2"/>
       <c r="AR2"/>
       <c r="AS2"/>
@@ -2286,64 +2341,64 @@
       <c r="AU2"/>
       <c r="AV2"/>
       <c r="AW2"/>
-      <c r="AX2" s="3" t="inlineStr">
+      <c r="AX2"/>
+      <c r="AY2"/>
+      <c r="AZ2"/>
+      <c r="BA2" s="3" t="inlineStr">
         <is>
           <t>351</t>
         </is>
       </c>
-      <c r="AY2" s="4" t="n">
+      <c r="BB2" s="4" t="n">
         <v>35930.0</v>
       </c>
-      <c r="AZ2"/>
-      <c r="BA2"/>
-      <c r="BB2"/>
       <c r="BC2"/>
       <c r="BD2"/>
       <c r="BE2"/>
       <c r="BF2"/>
       <c r="BG2"/>
-      <c r="BH2" s="3" t="inlineStr">
+      <c r="BH2"/>
+      <c r="BI2"/>
+      <c r="BJ2"/>
+      <c r="BK2" s="3" t="inlineStr">
         <is>
           <t>INSURED_SUBSCRIBER</t>
         </is>
       </c>
-      <c r="BI2" s="3" t="inlineStr">
+      <c r="BL2" s="3" t="inlineStr">
         <is>
           <t>SSN</t>
         </is>
       </c>
-      <c r="BJ2" s="3" t="inlineStr">
+      <c r="BM2" s="3" t="inlineStr">
         <is>
           <t>103229876</t>
         </is>
       </c>
-      <c r="BK2"/>
-      <c r="BL2" s="3" t="inlineStr">
+      <c r="BN2"/>
+      <c r="BO2" s="3" t="inlineStr">
         <is>
           <t>DOE</t>
         </is>
       </c>
-      <c r="BM2" s="3" t="inlineStr">
+      <c r="BP2" s="3" t="inlineStr">
         <is>
           <t>JAMES</t>
         </is>
       </c>
-      <c r="BN2" s="3" t="inlineStr">
+      <c r="BQ2" s="3" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="BO2" s="4" t="n">
+      <c r="BR2" s="4" t="n">
         <v>28353.0</v>
       </c>
-      <c r="BP2" s="3" t="inlineStr">
+      <c r="BS2" s="3" t="inlineStr">
         <is>
           <t>MALE</t>
         </is>
       </c>
-      <c r="BQ2"/>
-      <c r="BR2"/>
-      <c r="BS2"/>
       <c r="BT2"/>
       <c r="BU2"/>
       <c r="BV2"/>
@@ -2421,16 +2476,16 @@
       <c r="EP2"/>
       <c r="EQ2"/>
       <c r="ER2"/>
-      <c r="ES2" s="3" t="inlineStr">
-        <is>
-          <t>PENN STATE UNIVERSITY</t>
-        </is>
-      </c>
+      <c r="ES2"/>
       <c r="ET2"/>
       <c r="EU2"/>
       <c r="EV2"/>
       <c r="EW2"/>
-      <c r="EX2"/>
+      <c r="EX2" s="3" t="inlineStr">
+        <is>
+          <t>PENN STATE UNIVERSITY</t>
+        </is>
+      </c>
       <c r="EY2"/>
       <c r="EZ2"/>
       <c r="FA2"/>
@@ -2539,32 +2594,32 @@
       <c r="IZ2"/>
       <c r="JA2"/>
       <c r="JB2"/>
-      <c r="JC2" s="3" t="inlineStr">
-        <is>
-          <t>021</t>
-        </is>
-      </c>
-      <c r="JD2" s="3" t="inlineStr">
-        <is>
-          <t>HLT</t>
-        </is>
-      </c>
+      <c r="JC2"/>
+      <c r="JD2"/>
       <c r="JE2"/>
       <c r="JF2"/>
       <c r="JG2"/>
       <c r="JH2" s="3" t="inlineStr">
         <is>
-          <t>348</t>
-        </is>
-      </c>
-      <c r="JI2" s="4" t="n">
-        <v>35217.0</v>
+          <t>021</t>
+        </is>
+      </c>
+      <c r="JI2" s="3" t="inlineStr">
+        <is>
+          <t>HLT</t>
+        </is>
       </c>
       <c r="JJ2"/>
       <c r="JK2"/>
       <c r="JL2"/>
-      <c r="JM2"/>
-      <c r="JN2"/>
+      <c r="JM2" s="3" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="JN2" s="4" t="n">
+        <v>35217.0</v>
+      </c>
       <c r="JO2"/>
       <c r="JP2"/>
       <c r="JQ2"/>
@@ -2711,6 +2766,17 @@
       <c r="PB2"/>
       <c r="PC2"/>
       <c r="PD2"/>
+      <c r="PE2"/>
+      <c r="PF2"/>
+      <c r="PG2"/>
+      <c r="PH2"/>
+      <c r="PI2"/>
+      <c r="PJ2"/>
+      <c r="PK2"/>
+      <c r="PL2"/>
+      <c r="PM2"/>
+      <c r="PN2"/>
+      <c r="PO2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>